<commit_message>
Elv: tabela de espécies
</commit_message>
<xml_diff>
--- a/res/tabela da comunidade.xlsx
+++ b/res/tabela da comunidade.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_B992312702B166F0E476389F13FD156A6ADA3413" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED89D97A-0757-40C1-8C82-90E4A58F0585}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_B992312702B166F0E476389F13FD156A6ADA3413" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6581421A-5591-4556-A5C5-D1B7D845147B}"/>
   <bookViews>
-    <workbookView xWindow="-21600" yWindow="-12465" windowWidth="22335" windowHeight="27945" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3658" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3666" uniqueCount="182">
   <si>
     <t>Variable</t>
   </si>
@@ -501,6 +501,72 @@
   </si>
   <si>
     <t>Tri.tetractis</t>
+  </si>
+  <si>
+    <t>Stream</t>
+  </si>
+  <si>
+    <t>Season</t>
+  </si>
+  <si>
+    <t>Wet</t>
+  </si>
+  <si>
+    <t>Dry</t>
+  </si>
+  <si>
+    <t>Ponto10</t>
+  </si>
+  <si>
+    <t>Ponto5</t>
+  </si>
+  <si>
+    <t>Ponto6</t>
+  </si>
+  <si>
+    <t>Ponto7</t>
+  </si>
+  <si>
+    <t>Ponto8</t>
+  </si>
+  <si>
+    <t>Ponto9</t>
+  </si>
+  <si>
+    <t>Ponto12</t>
+  </si>
+  <si>
+    <t>Ponto13</t>
+  </si>
+  <si>
+    <t>Ponto14</t>
+  </si>
+  <si>
+    <t>Ponto15</t>
+  </si>
+  <si>
+    <t>Ponto16</t>
+  </si>
+  <si>
+    <t>Ponto17</t>
+  </si>
+  <si>
+    <t>Ponto18</t>
+  </si>
+  <si>
+    <t>Ponto19</t>
+  </si>
+  <si>
+    <t>Ponto20</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Barro Branco Stream</t>
+  </si>
+  <si>
+    <t>Caiana Stream</t>
   </si>
 </sst>
 </file>
@@ -536,8 +602,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,6 +628,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6450,300 +6529,192 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{768C672F-8BDD-430E-9621-0F0E0D5E9FE7}">
-  <dimension ref="A1:AE59"/>
+  <dimension ref="A1:AE61"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>30</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
+      <c r="AC1" s="3"/>
+      <c r="AD1" s="3"/>
+      <c r="AE1" s="3"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L2" t="s">
-        <v>35</v>
-      </c>
-      <c r="M2" t="s">
-        <v>33</v>
-      </c>
-      <c r="N2" t="s">
-        <v>36</v>
-      </c>
-      <c r="O2" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>33</v>
-      </c>
-      <c r="R2" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" t="s">
-        <v>38</v>
-      </c>
-      <c r="T2" t="s">
-        <v>36</v>
-      </c>
-      <c r="U2" t="s">
-        <v>33</v>
-      </c>
-      <c r="V2" t="s">
-        <v>33</v>
-      </c>
-      <c r="W2" t="s">
-        <v>33</v>
-      </c>
-      <c r="X2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>33</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>179</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>165</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>166</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>167</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>168</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>169</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>164</v>
       </c>
       <c r="H3" t="s">
-        <v>33</v>
+        <v>165</v>
       </c>
       <c r="I3" t="s">
-        <v>33</v>
+        <v>166</v>
       </c>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>167</v>
       </c>
       <c r="K3" t="s">
-        <v>33</v>
+        <v>168</v>
       </c>
       <c r="L3" t="s">
-        <v>33</v>
+        <v>169</v>
       </c>
       <c r="M3" t="s">
-        <v>33</v>
+        <v>164</v>
       </c>
       <c r="N3" t="s">
-        <v>33</v>
+        <v>170</v>
       </c>
       <c r="O3" t="s">
-        <v>33</v>
+        <v>171</v>
       </c>
       <c r="P3" t="s">
-        <v>33</v>
+        <v>172</v>
       </c>
       <c r="Q3" t="s">
-        <v>33</v>
+        <v>173</v>
       </c>
       <c r="R3" t="s">
-        <v>41</v>
+        <v>174</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>175</v>
       </c>
       <c r="T3" t="s">
-        <v>33</v>
+        <v>176</v>
       </c>
       <c r="U3" t="s">
-        <v>36</v>
+        <v>177</v>
       </c>
       <c r="V3" t="s">
-        <v>33</v>
+        <v>178</v>
       </c>
       <c r="W3" t="s">
-        <v>33</v>
+        <v>170</v>
       </c>
       <c r="X3" t="s">
-        <v>33</v>
+        <v>171</v>
       </c>
       <c r="Y3" t="s">
-        <v>33</v>
+        <v>172</v>
       </c>
       <c r="Z3" t="s">
-        <v>33</v>
+        <v>173</v>
       </c>
       <c r="AA3" t="s">
-        <v>33</v>
+        <v>174</v>
       </c>
       <c r="AB3" t="s">
-        <v>33</v>
+        <v>175</v>
       </c>
       <c r="AC3" t="s">
-        <v>33</v>
+        <v>176</v>
       </c>
       <c r="AD3" t="s">
-        <v>33</v>
+        <v>177</v>
       </c>
       <c r="AE3" t="s">
-        <v>33</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
         <v>33</v>
@@ -6752,13 +6723,13 @@
         <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
         <v>33</v>
@@ -6770,7 +6741,7 @@
         <v>33</v>
       </c>
       <c r="K4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L4" t="s">
         <v>33</v>
@@ -6779,25 +6750,25 @@
         <v>33</v>
       </c>
       <c r="N4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="P4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q4" t="s">
         <v>33</v>
       </c>
       <c r="R4" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="T4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U4" t="s">
         <v>33</v>
@@ -6835,102 +6806,102 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="J5" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="K5" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="L5" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="M5" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="N5" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="O5" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="P5" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="Q5" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="R5" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="S5" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="T5" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="U5" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="V5" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="W5" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="X5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Y5" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="Z5" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="AA5" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="AB5" t="s">
-        <v>67</v>
+        <v>33</v>
       </c>
       <c r="AC5" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="AD5" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="AE5" t="s">
-        <v>66</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -6942,13 +6913,13 @@
         <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
         <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
         <v>33</v>
@@ -6981,10 +6952,10 @@
         <v>33</v>
       </c>
       <c r="R6" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="S6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="T6" t="s">
         <v>33</v>
@@ -7025,102 +6996,102 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H7" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="I7" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="J7" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="K7" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="L7" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="M7" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="O7" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="P7" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="Q7" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="R7" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="S7" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="T7" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="U7" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="V7" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="W7" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="X7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Y7" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="Z7" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="AA7" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="AB7" t="s">
-        <v>33</v>
+        <v>67</v>
       </c>
       <c r="AC7" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="AD7" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="AE7" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
         <v>33</v>
@@ -7171,10 +7142,10 @@
         <v>33</v>
       </c>
       <c r="R8" t="s">
+        <v>55</v>
+      </c>
+      <c r="S8" t="s">
         <v>35</v>
-      </c>
-      <c r="S8" t="s">
-        <v>33</v>
       </c>
       <c r="T8" t="s">
         <v>33</v>
@@ -7215,25 +7186,25 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H9" t="s">
         <v>33</v>
@@ -7248,31 +7219,31 @@
         <v>33</v>
       </c>
       <c r="L9" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="M9" t="s">
         <v>33</v>
       </c>
       <c r="N9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O9" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="P9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Q9" t="s">
         <v>33</v>
       </c>
       <c r="R9" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
       <c r="S9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T9" t="s">
-        <v>83</v>
+        <v>33</v>
       </c>
       <c r="U9" t="s">
         <v>33</v>
@@ -7281,7 +7252,7 @@
         <v>33</v>
       </c>
       <c r="W9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="X9" t="s">
         <v>33</v>
@@ -7290,30 +7261,30 @@
         <v>33</v>
       </c>
       <c r="Z9" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="AA9" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AB9" t="s">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="AC9" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="AD9" t="s">
         <v>33</v>
       </c>
       <c r="AE9" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -7325,7 +7296,7 @@
         <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="G10" t="s">
         <v>33</v>
@@ -7361,13 +7332,13 @@
         <v>33</v>
       </c>
       <c r="R10" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="S10" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="T10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="U10" t="s">
         <v>33</v>
@@ -7405,25 +7376,25 @@
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="F11" t="s">
         <v>33</v>
       </c>
       <c r="G11" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="H11" t="s">
         <v>33</v>
@@ -7435,7 +7406,7 @@
         <v>33</v>
       </c>
       <c r="K11" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="L11" t="s">
         <v>33</v>
@@ -7444,25 +7415,25 @@
         <v>33</v>
       </c>
       <c r="N11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O11" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="P11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q11" t="s">
         <v>33</v>
       </c>
       <c r="R11" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="S11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T11" t="s">
-        <v>33</v>
+        <v>83</v>
       </c>
       <c r="U11" t="s">
         <v>33</v>
@@ -7471,7 +7442,7 @@
         <v>33</v>
       </c>
       <c r="W11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="X11" t="s">
         <v>33</v>
@@ -7480,30 +7451,30 @@
         <v>33</v>
       </c>
       <c r="Z11" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="AA11" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="AB11" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="AC11" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="AD11" t="s">
         <v>33</v>
       </c>
       <c r="AE11" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
         <v>33</v>
@@ -7512,13 +7483,13 @@
         <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="H12" t="s">
         <v>33</v>
@@ -7545,7 +7516,7 @@
         <v>33</v>
       </c>
       <c r="P12" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="Q12" t="s">
         <v>33</v>
@@ -7554,11 +7525,11 @@
         <v>88</v>
       </c>
       <c r="S12" t="s">
+        <v>41</v>
+      </c>
+      <c r="T12" t="s">
         <v>35</v>
       </c>
-      <c r="T12" t="s">
-        <v>41</v>
-      </c>
       <c r="U12" t="s">
         <v>33</v>
       </c>
@@ -7578,7 +7549,7 @@
         <v>33</v>
       </c>
       <c r="AA12" t="s">
-        <v>91</v>
+        <v>33</v>
       </c>
       <c r="AB12" t="s">
         <v>33</v>
@@ -7595,7 +7566,7 @@
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
         <v>33</v>
@@ -7673,7 +7644,7 @@
         <v>33</v>
       </c>
       <c r="AA13" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="AB13" t="s">
         <v>33</v>
@@ -7690,7 +7661,7 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
         <v>33</v>
@@ -7702,13 +7673,13 @@
         <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F14" t="s">
         <v>33</v>
       </c>
       <c r="G14" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H14" t="s">
         <v>33</v>
@@ -7735,19 +7706,19 @@
         <v>33</v>
       </c>
       <c r="P14" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Q14" t="s">
         <v>33</v>
       </c>
       <c r="R14" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="S14" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T14" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="U14" t="s">
         <v>33</v>
@@ -7768,7 +7739,7 @@
         <v>33</v>
       </c>
       <c r="AA14" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="AB14" t="s">
         <v>33</v>
@@ -7785,7 +7756,7 @@
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -7863,7 +7834,7 @@
         <v>33</v>
       </c>
       <c r="AA15" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="AB15" t="s">
         <v>33</v>
@@ -7880,7 +7851,7 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
         <v>33</v>
@@ -7975,10 +7946,10 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
         <v>33</v>
@@ -8026,7 +7997,7 @@
         <v>33</v>
       </c>
       <c r="R17" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="S17" t="s">
         <v>33</v>
@@ -8070,7 +8041,7 @@
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
@@ -8121,10 +8092,10 @@
         <v>33</v>
       </c>
       <c r="R18" t="s">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="S18" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="T18" t="s">
         <v>33</v>
@@ -8165,7 +8136,7 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
         <v>33</v>
@@ -8180,13 +8151,13 @@
         <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H19" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="I19" t="s">
         <v>33</v>
@@ -8198,7 +8169,7 @@
         <v>33</v>
       </c>
       <c r="L19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="M19" t="s">
         <v>33</v>
@@ -8216,7 +8187,7 @@
         <v>33</v>
       </c>
       <c r="R19" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="S19" t="s">
         <v>33</v>
@@ -8231,7 +8202,7 @@
         <v>33</v>
       </c>
       <c r="W19" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="X19" t="s">
         <v>33</v>
@@ -8243,7 +8214,7 @@
         <v>33</v>
       </c>
       <c r="AA19" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="AB19" t="s">
         <v>33</v>
@@ -8260,7 +8231,7 @@
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -8311,7 +8282,7 @@
         <v>33</v>
       </c>
       <c r="R20" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="S20" t="s">
         <v>35</v>
@@ -8355,7 +8326,7 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
@@ -8367,7 +8338,7 @@
         <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F21" t="s">
         <v>33</v>
@@ -8376,7 +8347,7 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="I21" t="s">
         <v>33</v>
@@ -8385,13 +8356,13 @@
         <v>33</v>
       </c>
       <c r="K21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L21" t="s">
         <v>33</v>
       </c>
       <c r="M21" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="N21" t="s">
         <v>33</v>
@@ -8406,34 +8377,34 @@
         <v>33</v>
       </c>
       <c r="R21" t="s">
+        <v>38</v>
+      </c>
+      <c r="S21" t="s">
+        <v>33</v>
+      </c>
+      <c r="T21" t="s">
+        <v>33</v>
+      </c>
+      <c r="U21" t="s">
+        <v>33</v>
+      </c>
+      <c r="V21" t="s">
+        <v>33</v>
+      </c>
+      <c r="W21" t="s">
+        <v>36</v>
+      </c>
+      <c r="X21" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA21" t="s">
         <v>35</v>
-      </c>
-      <c r="S21" t="s">
-        <v>33</v>
-      </c>
-      <c r="T21" t="s">
-        <v>33</v>
-      </c>
-      <c r="U21" t="s">
-        <v>33</v>
-      </c>
-      <c r="V21" t="s">
-        <v>33</v>
-      </c>
-      <c r="W21" t="s">
-        <v>33</v>
-      </c>
-      <c r="X21" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>33</v>
       </c>
       <c r="AB21" t="s">
         <v>33</v>
@@ -8450,7 +8421,7 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
         <v>33</v>
@@ -8501,7 +8472,7 @@
         <v>33</v>
       </c>
       <c r="R22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="S22" t="s">
         <v>35</v>
@@ -8545,7 +8516,7 @@
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B23" t="s">
         <v>33</v>
@@ -8581,7 +8552,7 @@
         <v>33</v>
       </c>
       <c r="M23" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="N23" t="s">
         <v>33</v>
@@ -8596,7 +8567,7 @@
         <v>33</v>
       </c>
       <c r="R23" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="S23" t="s">
         <v>33</v>
@@ -8640,7 +8611,7 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
@@ -8691,10 +8662,10 @@
         <v>33</v>
       </c>
       <c r="R24" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="S24" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T24" t="s">
         <v>33</v>
@@ -8735,10 +8706,10 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -8750,7 +8721,7 @@
         <v>33</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="G25" t="s">
         <v>33</v>
@@ -8786,7 +8757,7 @@
         <v>33</v>
       </c>
       <c r="R25" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S25" t="s">
         <v>33</v>
@@ -8830,7 +8801,7 @@
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B26" t="s">
         <v>33</v>
@@ -8875,16 +8846,16 @@
         <v>33</v>
       </c>
       <c r="P26" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="Q26" t="s">
         <v>33</v>
       </c>
       <c r="R26" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="S26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="T26" t="s">
         <v>33</v>
@@ -8925,7 +8896,7 @@
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -8937,13 +8908,13 @@
         <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="F27" t="s">
         <v>33</v>
       </c>
       <c r="G27" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="H27" t="s">
         <v>33</v>
@@ -8958,7 +8929,7 @@
         <v>33</v>
       </c>
       <c r="L27" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="M27" t="s">
         <v>33</v>
@@ -8976,10 +8947,10 @@
         <v>33</v>
       </c>
       <c r="R27" t="s">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="S27" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="T27" t="s">
         <v>33</v>
@@ -9020,7 +8991,7 @@
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B28" t="s">
         <v>33</v>
@@ -9065,16 +9036,16 @@
         <v>33</v>
       </c>
       <c r="P28" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Q28" t="s">
         <v>33</v>
       </c>
       <c r="R28" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="S28" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="T28" t="s">
         <v>33</v>
@@ -9115,7 +9086,7 @@
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B29" t="s">
         <v>33</v>
@@ -9145,7 +9116,7 @@
         <v>33</v>
       </c>
       <c r="K29" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L29" t="s">
         <v>33</v>
@@ -9166,10 +9137,10 @@
         <v>33</v>
       </c>
       <c r="R29" t="s">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="S29" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="T29" t="s">
         <v>33</v>
@@ -9210,7 +9181,7 @@
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B30" t="s">
         <v>33</v>
@@ -9261,7 +9232,7 @@
         <v>33</v>
       </c>
       <c r="R30" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="S30" t="s">
         <v>33</v>
@@ -9305,7 +9276,7 @@
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B31" t="s">
         <v>33</v>
@@ -9400,7 +9371,7 @@
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
@@ -9451,7 +9422,7 @@
         <v>33</v>
       </c>
       <c r="R32" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="S32" t="s">
         <v>33</v>
@@ -9495,7 +9466,7 @@
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
         <v>33</v>
@@ -9546,7 +9517,7 @@
         <v>33</v>
       </c>
       <c r="R33" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="S33" t="s">
         <v>33</v>
@@ -9590,7 +9561,7 @@
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
         <v>33</v>
@@ -9685,7 +9656,7 @@
     </row>
     <row r="35" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B35" t="s">
         <v>33</v>
@@ -9736,7 +9707,7 @@
         <v>33</v>
       </c>
       <c r="R35" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="S35" t="s">
         <v>33</v>
@@ -9780,7 +9751,7 @@
     </row>
     <row r="36" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
         <v>33</v>
@@ -9801,7 +9772,7 @@
         <v>33</v>
       </c>
       <c r="H36" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I36" t="s">
         <v>33</v>
@@ -9875,7 +9846,7 @@
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B37" t="s">
         <v>33</v>
@@ -9970,7 +9941,7 @@
     </row>
     <row r="38" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B38" t="s">
         <v>33</v>
@@ -9985,7 +9956,7 @@
         <v>33</v>
       </c>
       <c r="F38" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
       <c r="G38" t="s">
         <v>33</v>
@@ -10006,7 +9977,7 @@
         <v>33</v>
       </c>
       <c r="M38" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="N38" t="s">
         <v>33</v>
@@ -10021,7 +9992,7 @@
         <v>33</v>
       </c>
       <c r="R38" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="S38" t="s">
         <v>33</v>
@@ -10065,7 +10036,7 @@
     </row>
     <row r="39" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B39" t="s">
         <v>33</v>
@@ -10080,7 +10051,7 @@
         <v>33</v>
       </c>
       <c r="F39" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="G39" t="s">
         <v>33</v>
@@ -10160,7 +10131,7 @@
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B40" t="s">
         <v>33</v>
@@ -10172,10 +10143,10 @@
         <v>33</v>
       </c>
       <c r="E40" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="F40" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G40" t="s">
         <v>33</v>
@@ -10211,7 +10182,7 @@
         <v>33</v>
       </c>
       <c r="R40" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="S40" t="s">
         <v>33</v>
@@ -10255,7 +10226,7 @@
     </row>
     <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B41" t="s">
         <v>33</v>
@@ -10267,7 +10238,7 @@
         <v>33</v>
       </c>
       <c r="E41" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F41" t="s">
         <v>33</v>
@@ -10350,7 +10321,7 @@
     </row>
     <row r="42" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
@@ -10362,10 +10333,10 @@
         <v>33</v>
       </c>
       <c r="E42" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F42" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G42" t="s">
         <v>33</v>
@@ -10401,7 +10372,7 @@
         <v>33</v>
       </c>
       <c r="R42" t="s">
-        <v>129</v>
+        <v>33</v>
       </c>
       <c r="S42" t="s">
         <v>33</v>
@@ -10445,7 +10416,7 @@
     </row>
     <row r="43" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B43" t="s">
         <v>33</v>
@@ -10460,7 +10431,7 @@
         <v>33</v>
       </c>
       <c r="F43" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G43" t="s">
         <v>33</v>
@@ -10496,10 +10467,10 @@
         <v>33</v>
       </c>
       <c r="R43" t="s">
-        <v>131</v>
+        <v>33</v>
       </c>
       <c r="S43" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="T43" t="s">
         <v>33</v>
@@ -10540,7 +10511,7 @@
     </row>
     <row r="44" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B44" t="s">
         <v>33</v>
@@ -10552,7 +10523,7 @@
         <v>33</v>
       </c>
       <c r="E44" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F44" t="s">
         <v>33</v>
@@ -10591,7 +10562,7 @@
         <v>33</v>
       </c>
       <c r="R44" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="S44" t="s">
         <v>33</v>
@@ -10635,7 +10606,7 @@
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B45" t="s">
         <v>33</v>
@@ -10647,7 +10618,7 @@
         <v>33</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F45" t="s">
         <v>33</v>
@@ -10686,10 +10657,10 @@
         <v>33</v>
       </c>
       <c r="R45" t="s">
-        <v>33</v>
+        <v>131</v>
       </c>
       <c r="S45" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="T45" t="s">
         <v>33</v>
@@ -10730,7 +10701,7 @@
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B46" t="s">
         <v>33</v>
@@ -10781,7 +10752,7 @@
         <v>33</v>
       </c>
       <c r="R46" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="S46" t="s">
         <v>33</v>
@@ -10825,7 +10796,7 @@
     </row>
     <row r="47" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B47" t="s">
         <v>33</v>
@@ -10920,31 +10891,31 @@
     </row>
     <row r="48" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B48" t="s">
-        <v>138</v>
+        <v>33</v>
       </c>
       <c r="C48" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F48" t="s">
-        <v>139</v>
+        <v>33</v>
       </c>
       <c r="G48" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="H48" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="I48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J48" t="s">
         <v>33</v>
@@ -10953,31 +10924,31 @@
         <v>33</v>
       </c>
       <c r="L48" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="M48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N48" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="O48" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="P48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="Q48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="R48" t="s">
-        <v>140</v>
+        <v>33</v>
       </c>
       <c r="S48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="T48" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="U48" t="s">
         <v>33</v>
@@ -10986,25 +10957,25 @@
         <v>33</v>
       </c>
       <c r="W48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="X48" t="s">
         <v>33</v>
       </c>
       <c r="Y48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="Z48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="AA48" t="s">
-        <v>141</v>
+        <v>33</v>
       </c>
       <c r="AB48" t="s">
-        <v>142</v>
+        <v>33</v>
       </c>
       <c r="AC48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AD48" t="s">
         <v>33</v>
@@ -11015,7 +10986,7 @@
     </row>
     <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B49" t="s">
         <v>33</v>
@@ -11066,13 +11037,13 @@
         <v>33</v>
       </c>
       <c r="R49" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="S49" t="s">
         <v>33</v>
       </c>
       <c r="T49" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="U49" t="s">
         <v>33</v>
@@ -11093,10 +11064,10 @@
         <v>33</v>
       </c>
       <c r="AA49" t="s">
-        <v>144</v>
+        <v>33</v>
       </c>
       <c r="AB49" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="AC49" t="s">
         <v>33</v>
@@ -11110,28 +11081,28 @@
     </row>
     <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B50" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D50" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E50" t="s">
-        <v>33</v>
+        <v>139</v>
       </c>
       <c r="F50" t="s">
-        <v>146</v>
+        <v>43</v>
       </c>
       <c r="G50" t="s">
-        <v>33</v>
+        <v>138</v>
       </c>
       <c r="H50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I50" t="s">
         <v>33</v>
@@ -11140,61 +11111,61 @@
         <v>33</v>
       </c>
       <c r="K50" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="L50" t="s">
+        <v>36</v>
+      </c>
+      <c r="M50" t="s">
+        <v>41</v>
+      </c>
+      <c r="N50" t="s">
+        <v>85</v>
+      </c>
+      <c r="O50" t="s">
+        <v>38</v>
+      </c>
+      <c r="P50" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>36</v>
+      </c>
+      <c r="R50" t="s">
+        <v>140</v>
+      </c>
+      <c r="S50" t="s">
         <v>35</v>
       </c>
-      <c r="M50" t="s">
-        <v>33</v>
-      </c>
-      <c r="N50" t="s">
-        <v>33</v>
-      </c>
-      <c r="O50" t="s">
-        <v>33</v>
-      </c>
-      <c r="P50" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q50" t="s">
-        <v>33</v>
-      </c>
-      <c r="R50" t="s">
-        <v>85</v>
-      </c>
-      <c r="S50" t="s">
-        <v>33</v>
-      </c>
       <c r="T50" t="s">
+        <v>110</v>
+      </c>
+      <c r="U50" t="s">
+        <v>33</v>
+      </c>
+      <c r="V50" t="s">
+        <v>33</v>
+      </c>
+      <c r="W50" t="s">
         <v>35</v>
       </c>
-      <c r="U50" t="s">
-        <v>33</v>
-      </c>
-      <c r="V50" t="s">
-        <v>33</v>
-      </c>
-      <c r="W50" t="s">
-        <v>33</v>
-      </c>
       <c r="X50" t="s">
         <v>33</v>
       </c>
       <c r="Y50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Z50" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AA50" t="s">
-        <v>35</v>
+        <v>141</v>
       </c>
       <c r="AB50" t="s">
-        <v>45</v>
+        <v>142</v>
       </c>
       <c r="AC50" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="AD50" t="s">
         <v>33</v>
@@ -11205,10 +11176,10 @@
     </row>
     <row r="51" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B51" t="s">
-        <v>148</v>
+        <v>33</v>
       </c>
       <c r="C51" t="s">
         <v>33</v>
@@ -11256,13 +11227,13 @@
         <v>33</v>
       </c>
       <c r="R51" t="s">
-        <v>149</v>
+        <v>38</v>
       </c>
       <c r="S51" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="T51" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U51" t="s">
         <v>33</v>
@@ -11283,10 +11254,10 @@
         <v>33</v>
       </c>
       <c r="AA51" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
       <c r="AB51" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AC51" t="s">
         <v>33</v>
@@ -11300,7 +11271,7 @@
     </row>
     <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B52" t="s">
         <v>33</v>
@@ -11312,7 +11283,7 @@
         <v>33</v>
       </c>
       <c r="E52" t="s">
-        <v>33</v>
+        <v>146</v>
       </c>
       <c r="F52" t="s">
         <v>33</v>
@@ -11330,13 +11301,13 @@
         <v>33</v>
       </c>
       <c r="K52" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L52" t="s">
         <v>33</v>
       </c>
       <c r="M52" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="N52" t="s">
         <v>33</v>
@@ -11351,13 +11322,13 @@
         <v>33</v>
       </c>
       <c r="R52" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="S52" t="s">
         <v>33</v>
       </c>
       <c r="T52" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="U52" t="s">
         <v>33</v>
@@ -11378,10 +11349,10 @@
         <v>33</v>
       </c>
       <c r="AA52" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AB52" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="AC52" t="s">
         <v>33</v>
@@ -11395,7 +11366,7 @@
     </row>
     <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B53" t="s">
         <v>33</v>
@@ -11413,7 +11384,7 @@
         <v>33</v>
       </c>
       <c r="G53" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
       <c r="H53" t="s">
         <v>33</v>
@@ -11446,13 +11417,13 @@
         <v>33</v>
       </c>
       <c r="R53" t="s">
-        <v>33</v>
+        <v>149</v>
       </c>
       <c r="S53" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="T53" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U53" t="s">
         <v>33</v>
@@ -11473,7 +11444,7 @@
         <v>33</v>
       </c>
       <c r="AA53" t="s">
-        <v>91</v>
+        <v>33</v>
       </c>
       <c r="AB53" t="s">
         <v>33</v>
@@ -11490,7 +11461,7 @@
     </row>
     <row r="54" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B54" t="s">
         <v>33</v>
@@ -11523,7 +11494,7 @@
         <v>33</v>
       </c>
       <c r="L54" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="M54" t="s">
         <v>33</v>
@@ -11585,7 +11556,7 @@
     </row>
     <row r="55" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B55" t="s">
         <v>33</v>
@@ -11663,7 +11634,7 @@
         <v>33</v>
       </c>
       <c r="AA55" t="s">
-        <v>154</v>
+        <v>91</v>
       </c>
       <c r="AB55" t="s">
         <v>33</v>
@@ -11680,7 +11651,7 @@
     </row>
     <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B56" t="s">
         <v>33</v>
@@ -11731,10 +11702,10 @@
         <v>33</v>
       </c>
       <c r="R56" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="S56" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="T56" t="s">
         <v>33</v>
@@ -11758,7 +11729,7 @@
         <v>33</v>
       </c>
       <c r="AA56" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="AB56" t="s">
         <v>33</v>
@@ -11775,7 +11746,7 @@
     </row>
     <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B57" t="s">
         <v>33</v>
@@ -11826,7 +11797,7 @@
         <v>33</v>
       </c>
       <c r="R57" t="s">
-        <v>157</v>
+        <v>33</v>
       </c>
       <c r="S57" t="s">
         <v>33</v>
@@ -11853,7 +11824,7 @@
         <v>33</v>
       </c>
       <c r="AA57" t="s">
-        <v>33</v>
+        <v>154</v>
       </c>
       <c r="AB57" t="s">
         <v>33</v>
@@ -11870,7 +11841,7 @@
     </row>
     <row r="58" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B58" t="s">
         <v>33</v>
@@ -11921,10 +11892,10 @@
         <v>33</v>
       </c>
       <c r="R58" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="S58" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="T58" t="s">
         <v>33</v>
@@ -11948,7 +11919,7 @@
         <v>33</v>
       </c>
       <c r="AA58" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AB58" t="s">
         <v>33</v>
@@ -11965,100 +11936,296 @@
     </row>
     <row r="59" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>156</v>
+      </c>
+      <c r="B59" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" t="s">
+        <v>33</v>
+      </c>
+      <c r="D59" t="s">
+        <v>33</v>
+      </c>
+      <c r="E59" t="s">
+        <v>33</v>
+      </c>
+      <c r="F59" t="s">
+        <v>33</v>
+      </c>
+      <c r="G59" t="s">
+        <v>33</v>
+      </c>
+      <c r="H59" t="s">
+        <v>33</v>
+      </c>
+      <c r="I59" t="s">
+        <v>33</v>
+      </c>
+      <c r="J59" t="s">
+        <v>33</v>
+      </c>
+      <c r="K59" t="s">
+        <v>33</v>
+      </c>
+      <c r="L59" t="s">
+        <v>33</v>
+      </c>
+      <c r="M59" t="s">
+        <v>33</v>
+      </c>
+      <c r="N59" t="s">
+        <v>33</v>
+      </c>
+      <c r="O59" t="s">
+        <v>33</v>
+      </c>
+      <c r="P59" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>33</v>
+      </c>
+      <c r="R59" t="s">
+        <v>157</v>
+      </c>
+      <c r="S59" t="s">
+        <v>33</v>
+      </c>
+      <c r="T59" t="s">
+        <v>33</v>
+      </c>
+      <c r="U59" t="s">
+        <v>33</v>
+      </c>
+      <c r="V59" t="s">
+        <v>33</v>
+      </c>
+      <c r="W59" t="s">
+        <v>33</v>
+      </c>
+      <c r="X59" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y59" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z59" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA59" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB59" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC59" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD59" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE59" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>158</v>
+      </c>
+      <c r="B60" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" t="s">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s">
+        <v>33</v>
+      </c>
+      <c r="F60" t="s">
+        <v>33</v>
+      </c>
+      <c r="G60" t="s">
+        <v>33</v>
+      </c>
+      <c r="H60" t="s">
+        <v>33</v>
+      </c>
+      <c r="I60" t="s">
+        <v>33</v>
+      </c>
+      <c r="J60" t="s">
+        <v>33</v>
+      </c>
+      <c r="K60" t="s">
+        <v>33</v>
+      </c>
+      <c r="L60" t="s">
+        <v>33</v>
+      </c>
+      <c r="M60" t="s">
+        <v>33</v>
+      </c>
+      <c r="N60" t="s">
+        <v>33</v>
+      </c>
+      <c r="O60" t="s">
+        <v>33</v>
+      </c>
+      <c r="P60" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>33</v>
+      </c>
+      <c r="R60" t="s">
+        <v>33</v>
+      </c>
+      <c r="S60" t="s">
+        <v>33</v>
+      </c>
+      <c r="T60" t="s">
+        <v>33</v>
+      </c>
+      <c r="U60" t="s">
+        <v>33</v>
+      </c>
+      <c r="V60" t="s">
+        <v>33</v>
+      </c>
+      <c r="W60" t="s">
+        <v>33</v>
+      </c>
+      <c r="X60" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y60" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z60" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA60" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB60" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC60" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD60" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE60" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>159</v>
       </c>
-      <c r="B59" t="s">
-        <v>33</v>
-      </c>
-      <c r="C59" t="s">
-        <v>33</v>
-      </c>
-      <c r="D59" t="s">
-        <v>33</v>
-      </c>
-      <c r="E59" t="s">
-        <v>33</v>
-      </c>
-      <c r="F59" t="s">
-        <v>33</v>
-      </c>
-      <c r="G59" t="s">
-        <v>33</v>
-      </c>
-      <c r="H59" t="s">
-        <v>33</v>
-      </c>
-      <c r="I59" t="s">
-        <v>33</v>
-      </c>
-      <c r="J59" t="s">
-        <v>33</v>
-      </c>
-      <c r="K59" t="s">
-        <v>33</v>
-      </c>
-      <c r="L59" t="s">
-        <v>33</v>
-      </c>
-      <c r="M59" t="s">
-        <v>33</v>
-      </c>
-      <c r="N59" t="s">
-        <v>33</v>
-      </c>
-      <c r="O59" t="s">
-        <v>33</v>
-      </c>
-      <c r="P59" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q59" t="s">
-        <v>33</v>
-      </c>
-      <c r="R59" t="s">
-        <v>33</v>
-      </c>
-      <c r="S59" t="s">
-        <v>33</v>
-      </c>
-      <c r="T59" t="s">
-        <v>33</v>
-      </c>
-      <c r="U59" t="s">
-        <v>33</v>
-      </c>
-      <c r="V59" t="s">
-        <v>33</v>
-      </c>
-      <c r="W59" t="s">
-        <v>33</v>
-      </c>
-      <c r="X59" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y59" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z59" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA59" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB59" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC59" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD59" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE59" t="s">
+      <c r="B61" t="s">
+        <v>33</v>
+      </c>
+      <c r="C61" t="s">
+        <v>33</v>
+      </c>
+      <c r="D61" t="s">
+        <v>33</v>
+      </c>
+      <c r="E61" t="s">
+        <v>33</v>
+      </c>
+      <c r="F61" t="s">
+        <v>33</v>
+      </c>
+      <c r="G61" t="s">
+        <v>33</v>
+      </c>
+      <c r="H61" t="s">
+        <v>33</v>
+      </c>
+      <c r="I61" t="s">
+        <v>33</v>
+      </c>
+      <c r="J61" t="s">
+        <v>33</v>
+      </c>
+      <c r="K61" t="s">
+        <v>33</v>
+      </c>
+      <c r="L61" t="s">
+        <v>33</v>
+      </c>
+      <c r="M61" t="s">
+        <v>33</v>
+      </c>
+      <c r="N61" t="s">
+        <v>33</v>
+      </c>
+      <c r="O61" t="s">
+        <v>33</v>
+      </c>
+      <c r="P61" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>33</v>
+      </c>
+      <c r="R61" t="s">
+        <v>33</v>
+      </c>
+      <c r="S61" t="s">
+        <v>33</v>
+      </c>
+      <c r="T61" t="s">
+        <v>33</v>
+      </c>
+      <c r="U61" t="s">
+        <v>33</v>
+      </c>
+      <c r="V61" t="s">
+        <v>33</v>
+      </c>
+      <c r="W61" t="s">
+        <v>33</v>
+      </c>
+      <c r="X61" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y61" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z61" t="s">
+        <v>33</v>
+      </c>
+      <c r="AA61" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB61" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC61" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD61" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE61" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="N2:V2"/>
+    <mergeCell ref="W2:AE2"/>
+  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>